<commit_message>
docs(demo): add public fixture proof package
</commit_message>
<xml_diff>
--- a/output/demo/demo-workbook.xlsx
+++ b/output/demo/demo-workbook.xlsx
@@ -1,92 +1,92 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Queue" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Explorer" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Hotspots" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operator Outcomes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approval Ledger" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Intelligence" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo Detail" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Lens" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Collection" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trend Summary" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Changes" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaigns" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance Controls" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Pack" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Items" sheetId="18" state="hidden" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity" sheetId="19" state="hidden" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Repos" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Badges" sheetId="21" state="hidden" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="22" state="hidden" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compare" sheetId="23" state="hidden" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_ActionSyncAutomation" sheetId="24" state="hidden" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_ActionSyncOutcomes" sheetId="25" state="hidden" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Actions" sheetId="26" state="hidden" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_ApprovalLedger" sheetId="27" state="hidden" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_CampaignTuning" sheetId="28" state="hidden" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Campaigns" sheetId="29" state="hidden" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Collections" sheetId="30" state="hidden" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Dimensions" sheetId="31" state="hidden" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Governance" sheetId="32" state="hidden" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_History" sheetId="33" state="hidden" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_ImplementationHotspots" sheetId="34" state="hidden" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_InterventionLedger" sheetId="35" state="hidden" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Lenses" sheetId="36" state="hidden" r:id="rId36"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_MaterialChangeRollups" sheetId="37" state="hidden" r:id="rId37"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_OperatorOutcomes" sheetId="38" state="hidden" r:id="rId38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_OperatorQueue" sheetId="39" state="hidden" r:id="rId39"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_OperatorRepoRollups" sheetId="40" state="hidden" r:id="rId40"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_PortfolioCatalog" sheetId="41" state="hidden" r:id="rId41"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_PortfolioHistory" sheetId="42" state="hidden" r:id="rId42"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_RepoDetail" sheetId="43" state="hidden" r:id="rId43"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_RepoDimensionRollups" sheetId="44" state="hidden" r:id="rId44"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_RepoHistoryRollups" sheetId="45" state="hidden" r:id="rId45"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Repos" sheetId="46" state="hidden" r:id="rId46"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_ReviewHistory" sheetId="47" state="hidden" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_ReviewTargets" sheetId="48" state="hidden" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Rollups" sheetId="49" state="hidden" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_RunChangeRepoData" sheetId="50" state="hidden" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_RunChangeRollups" sheetId="51" state="hidden" r:id="rId51"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Scenarios" sheetId="52" state="hidden" r:id="rId52"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Scorecards" sheetId="53" state="hidden" r:id="rId53"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Security" sheetId="54" state="hidden" r:id="rId54"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_SecurityAlerts" sheetId="55" state="hidden" r:id="rId55"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_SecurityControls" sheetId="56" state="hidden" r:id="rId56"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_SecurityProviders" sheetId="57" state="hidden" r:id="rId57"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_TrendMatrix" sheetId="58" state="hidden" r:id="rId58"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Writeback" sheetId="59" state="hidden" r:id="rId59"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dep Graph" sheetId="60" state="hidden" r:id="rId60"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance Audit" sheetId="61" state="hidden" r:id="rId61"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hotspots" sheetId="62" state="hidden" r:id="rId62"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Initiative Tracker" sheetId="63" state="hidden" r:id="rId63"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookups" sheetId="64" state="hidden" r:id="rId64"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Catalog" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Wins" sheetId="66" state="hidden" r:id="rId66"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo Profiles" sheetId="67" state="hidden" r:id="rId67"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review History" sheetId="68" state="hidden" r:id="rId68"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Planner" sheetId="69" state="hidden" r:id="rId69"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Score Explainer" sheetId="70" state="hidden" r:id="rId70"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorecards" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Heatmap" sheetId="72" state="hidden" r:id="rId72"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="73" state="hidden" r:id="rId73"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Controls" sheetId="74" state="hidden" r:id="rId74"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Debt" sheetId="75" state="hidden" r:id="rId75"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply Chain" sheetId="76" state="hidden" r:id="rId76"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TemplateInfo" sheetId="77" state="hidden" r:id="rId77"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier Breakdown" sheetId="78" state="hidden" r:id="rId78"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trends" sheetId="79" state="hidden" r:id="rId79"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Writeback Audit" sheetId="80" state="hidden" r:id="rId80"/>
+    <sheet name="Index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Review Queue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Portfolio Explorer" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Implementation Hotspots" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Operator Outcomes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Approval Ledger" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Historical Intelligence" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Repo Detail" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Executive Summary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="By Lens" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="By Collection" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Trend Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Run Changes" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Campaigns" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Governance Controls" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Print Pack" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Action Items" sheetId="18" state="hidden" r:id="rId18"/>
+    <sheet name="Activity" sheetId="19" state="hidden" r:id="rId19"/>
+    <sheet name="All Repos" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Badges" sheetId="21" state="hidden" r:id="rId21"/>
+    <sheet name="Changes" sheetId="22" state="hidden" r:id="rId22"/>
+    <sheet name="Compare" sheetId="23" state="hidden" r:id="rId23"/>
+    <sheet name="Data_ActionSyncAutomation" sheetId="24" state="hidden" r:id="rId24"/>
+    <sheet name="Data_ActionSyncOutcomes" sheetId="25" state="hidden" r:id="rId25"/>
+    <sheet name="Data_Actions" sheetId="26" state="hidden" r:id="rId26"/>
+    <sheet name="Data_ApprovalLedger" sheetId="27" state="hidden" r:id="rId27"/>
+    <sheet name="Data_CampaignTuning" sheetId="28" state="hidden" r:id="rId28"/>
+    <sheet name="Data_Campaigns" sheetId="29" state="hidden" r:id="rId29"/>
+    <sheet name="Data_Collections" sheetId="30" state="hidden" r:id="rId30"/>
+    <sheet name="Data_Dimensions" sheetId="31" state="hidden" r:id="rId31"/>
+    <sheet name="Data_Governance" sheetId="32" state="hidden" r:id="rId32"/>
+    <sheet name="Data_History" sheetId="33" state="hidden" r:id="rId33"/>
+    <sheet name="Data_ImplementationHotspots" sheetId="34" state="hidden" r:id="rId34"/>
+    <sheet name="Data_InterventionLedger" sheetId="35" state="hidden" r:id="rId35"/>
+    <sheet name="Data_Lenses" sheetId="36" state="hidden" r:id="rId36"/>
+    <sheet name="Data_MaterialChangeRollups" sheetId="37" state="hidden" r:id="rId37"/>
+    <sheet name="Data_OperatorOutcomes" sheetId="38" state="hidden" r:id="rId38"/>
+    <sheet name="Data_OperatorQueue" sheetId="39" state="hidden" r:id="rId39"/>
+    <sheet name="Data_OperatorRepoRollups" sheetId="40" state="hidden" r:id="rId40"/>
+    <sheet name="Data_PortfolioCatalog" sheetId="41" state="hidden" r:id="rId41"/>
+    <sheet name="Data_PortfolioHistory" sheetId="42" state="hidden" r:id="rId42"/>
+    <sheet name="Data_RepoDetail" sheetId="43" state="hidden" r:id="rId43"/>
+    <sheet name="Data_RepoDimensionRollups" sheetId="44" state="hidden" r:id="rId44"/>
+    <sheet name="Data_RepoHistoryRollups" sheetId="45" state="hidden" r:id="rId45"/>
+    <sheet name="Data_Repos" sheetId="46" state="hidden" r:id="rId46"/>
+    <sheet name="Data_ReviewHistory" sheetId="47" state="hidden" r:id="rId47"/>
+    <sheet name="Data_ReviewTargets" sheetId="48" state="hidden" r:id="rId48"/>
+    <sheet name="Data_Rollups" sheetId="49" state="hidden" r:id="rId49"/>
+    <sheet name="Data_RunChangeRepoData" sheetId="50" state="hidden" r:id="rId50"/>
+    <sheet name="Data_RunChangeRollups" sheetId="51" state="hidden" r:id="rId51"/>
+    <sheet name="Data_Scenarios" sheetId="52" state="hidden" r:id="rId52"/>
+    <sheet name="Data_Scorecards" sheetId="53" state="hidden" r:id="rId53"/>
+    <sheet name="Data_Security" sheetId="54" state="hidden" r:id="rId54"/>
+    <sheet name="Data_SecurityAlerts" sheetId="55" state="hidden" r:id="rId55"/>
+    <sheet name="Data_SecurityControls" sheetId="56" state="hidden" r:id="rId56"/>
+    <sheet name="Data_SecurityProviders" sheetId="57" state="hidden" r:id="rId57"/>
+    <sheet name="Data_TrendMatrix" sheetId="58" state="hidden" r:id="rId58"/>
+    <sheet name="Data_Writeback" sheetId="59" state="hidden" r:id="rId59"/>
+    <sheet name="Dep Graph" sheetId="60" state="hidden" r:id="rId60"/>
+    <sheet name="Governance Audit" sheetId="61" state="hidden" r:id="rId61"/>
+    <sheet name="Hotspots" sheetId="62" state="hidden" r:id="rId62"/>
+    <sheet name="Initiative Tracker" sheetId="63" state="hidden" r:id="rId63"/>
+    <sheet name="Lookups" sheetId="64" state="hidden" r:id="rId64"/>
+    <sheet name="Portfolio Catalog" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="Quick Wins" sheetId="66" state="hidden" r:id="rId66"/>
+    <sheet name="Repo Profiles" sheetId="67" state="hidden" r:id="rId67"/>
+    <sheet name="Review History" sheetId="68" state="hidden" r:id="rId68"/>
+    <sheet name="Scenario Planner" sheetId="69" state="hidden" r:id="rId69"/>
+    <sheet name="Score Explainer" sheetId="70" state="hidden" r:id="rId70"/>
+    <sheet name="Scorecards" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="Scoring Heatmap" sheetId="72" state="hidden" r:id="rId72"/>
+    <sheet name="Security" sheetId="73" state="hidden" r:id="rId73"/>
+    <sheet name="Security Controls" sheetId="74" state="hidden" r:id="rId74"/>
+    <sheet name="Security Debt" sheetId="75" state="hidden" r:id="rId75"/>
+    <sheet name="Supply Chain" sheetId="76" state="hidden" r:id="rId76"/>
+    <sheet name="TemplateInfo" sheetId="77" state="hidden" r:id="rId77"/>
+    <sheet name="Tier Breakdown" sheetId="78" state="hidden" r:id="rId78"/>
+    <sheet name="Trends" sheetId="79" state="hidden" r:id="rId79"/>
+    <sheet name="Writeback Audit" sheetId="80" state="hidden" r:id="rId80"/>
   </sheets>
   <definedNames>
     <definedName name="nrGeneratedAt">'Dashboard'!$A$2</definedName>
@@ -721,14 +721,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -746,17 +746,17 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <dPt>
             <idx val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="166534"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -764,10 +764,10 @@
           <dPt>
             <idx val="1"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="1565C0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -775,10 +775,10 @@
           <dPt>
             <idx val="2"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D97706"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -786,10 +786,10 @@
           <dPt>
             <idx val="3"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C2410C"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -797,10 +797,10 @@
           <dPt>
             <idx val="4"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="6B7280"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -833,14 +833,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -859,7 +859,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -911,14 +911,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -937,7 +937,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -989,14 +989,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1013,7 +1013,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1021,7 +1021,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1031,7 +1031,7 @@
           <idx val="1"/>
           <order val="1"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+            <a:ln w="12700">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -1041,7 +1041,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1051,7 +1051,7 @@
           <idx val="2"/>
           <order val="2"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+            <a:ln w="12700">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -1061,7 +1061,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1082,8 +1082,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1110,8 +1110,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1137,14 +1137,14 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1163,10 +1163,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="7C3AED"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1218,14 +1218,14 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="26"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1248,14 +1248,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1280,14 +1280,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1312,14 +1312,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1372,7 +1372,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -1387,9 +1387,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1409,9 +1409,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1431,9 +1431,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1453,9 +1453,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1465,7 +1465,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1480,9 +1480,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1492,7 +1492,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -1507,9 +1507,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
Add public-safe Portfolio Command Center fixture proof package (#120)
* docs(demo): add public fixture proof package

* fix(demo): keep fixture proof outputs isolated
</commit_message>
<xml_diff>
--- a/output/demo/demo-workbook.xlsx
+++ b/output/demo/demo-workbook.xlsx
@@ -1,92 +1,92 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Queue" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Explorer" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Hotspots" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operator Outcomes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approval Ledger" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Intelligence" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo Detail" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Lens" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Collection" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trend Summary" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Changes" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaigns" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance Controls" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Pack" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Items" sheetId="18" state="hidden" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity" sheetId="19" state="hidden" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Repos" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Badges" sheetId="21" state="hidden" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="22" state="hidden" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compare" sheetId="23" state="hidden" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_ActionSyncAutomation" sheetId="24" state="hidden" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_ActionSyncOutcomes" sheetId="25" state="hidden" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Actions" sheetId="26" state="hidden" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_ApprovalLedger" sheetId="27" state="hidden" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_CampaignTuning" sheetId="28" state="hidden" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Campaigns" sheetId="29" state="hidden" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Collections" sheetId="30" state="hidden" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Dimensions" sheetId="31" state="hidden" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Governance" sheetId="32" state="hidden" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_History" sheetId="33" state="hidden" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_ImplementationHotspots" sheetId="34" state="hidden" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_InterventionLedger" sheetId="35" state="hidden" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Lenses" sheetId="36" state="hidden" r:id="rId36"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_MaterialChangeRollups" sheetId="37" state="hidden" r:id="rId37"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_OperatorOutcomes" sheetId="38" state="hidden" r:id="rId38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_OperatorQueue" sheetId="39" state="hidden" r:id="rId39"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_OperatorRepoRollups" sheetId="40" state="hidden" r:id="rId40"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_PortfolioCatalog" sheetId="41" state="hidden" r:id="rId41"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_PortfolioHistory" sheetId="42" state="hidden" r:id="rId42"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_RepoDetail" sheetId="43" state="hidden" r:id="rId43"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_RepoDimensionRollups" sheetId="44" state="hidden" r:id="rId44"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_RepoHistoryRollups" sheetId="45" state="hidden" r:id="rId45"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Repos" sheetId="46" state="hidden" r:id="rId46"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_ReviewHistory" sheetId="47" state="hidden" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_ReviewTargets" sheetId="48" state="hidden" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Rollups" sheetId="49" state="hidden" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_RunChangeRepoData" sheetId="50" state="hidden" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_RunChangeRollups" sheetId="51" state="hidden" r:id="rId51"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Scenarios" sheetId="52" state="hidden" r:id="rId52"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Scorecards" sheetId="53" state="hidden" r:id="rId53"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Security" sheetId="54" state="hidden" r:id="rId54"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_SecurityAlerts" sheetId="55" state="hidden" r:id="rId55"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_SecurityControls" sheetId="56" state="hidden" r:id="rId56"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_SecurityProviders" sheetId="57" state="hidden" r:id="rId57"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_TrendMatrix" sheetId="58" state="hidden" r:id="rId58"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Writeback" sheetId="59" state="hidden" r:id="rId59"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dep Graph" sheetId="60" state="hidden" r:id="rId60"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance Audit" sheetId="61" state="hidden" r:id="rId61"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hotspots" sheetId="62" state="hidden" r:id="rId62"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Initiative Tracker" sheetId="63" state="hidden" r:id="rId63"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookups" sheetId="64" state="hidden" r:id="rId64"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Catalog" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Wins" sheetId="66" state="hidden" r:id="rId66"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo Profiles" sheetId="67" state="hidden" r:id="rId67"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review History" sheetId="68" state="hidden" r:id="rId68"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Planner" sheetId="69" state="hidden" r:id="rId69"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Score Explainer" sheetId="70" state="hidden" r:id="rId70"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorecards" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Heatmap" sheetId="72" state="hidden" r:id="rId72"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="73" state="hidden" r:id="rId73"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Controls" sheetId="74" state="hidden" r:id="rId74"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Debt" sheetId="75" state="hidden" r:id="rId75"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply Chain" sheetId="76" state="hidden" r:id="rId76"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TemplateInfo" sheetId="77" state="hidden" r:id="rId77"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier Breakdown" sheetId="78" state="hidden" r:id="rId78"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trends" sheetId="79" state="hidden" r:id="rId79"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Writeback Audit" sheetId="80" state="hidden" r:id="rId80"/>
+    <sheet name="Index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Review Queue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Portfolio Explorer" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Implementation Hotspots" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Operator Outcomes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Approval Ledger" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Historical Intelligence" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Repo Detail" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Executive Summary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="By Lens" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="By Collection" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Trend Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Run Changes" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Campaigns" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Governance Controls" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Print Pack" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Action Items" sheetId="18" state="hidden" r:id="rId18"/>
+    <sheet name="Activity" sheetId="19" state="hidden" r:id="rId19"/>
+    <sheet name="All Repos" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Badges" sheetId="21" state="hidden" r:id="rId21"/>
+    <sheet name="Changes" sheetId="22" state="hidden" r:id="rId22"/>
+    <sheet name="Compare" sheetId="23" state="hidden" r:id="rId23"/>
+    <sheet name="Data_ActionSyncAutomation" sheetId="24" state="hidden" r:id="rId24"/>
+    <sheet name="Data_ActionSyncOutcomes" sheetId="25" state="hidden" r:id="rId25"/>
+    <sheet name="Data_Actions" sheetId="26" state="hidden" r:id="rId26"/>
+    <sheet name="Data_ApprovalLedger" sheetId="27" state="hidden" r:id="rId27"/>
+    <sheet name="Data_CampaignTuning" sheetId="28" state="hidden" r:id="rId28"/>
+    <sheet name="Data_Campaigns" sheetId="29" state="hidden" r:id="rId29"/>
+    <sheet name="Data_Collections" sheetId="30" state="hidden" r:id="rId30"/>
+    <sheet name="Data_Dimensions" sheetId="31" state="hidden" r:id="rId31"/>
+    <sheet name="Data_Governance" sheetId="32" state="hidden" r:id="rId32"/>
+    <sheet name="Data_History" sheetId="33" state="hidden" r:id="rId33"/>
+    <sheet name="Data_ImplementationHotspots" sheetId="34" state="hidden" r:id="rId34"/>
+    <sheet name="Data_InterventionLedger" sheetId="35" state="hidden" r:id="rId35"/>
+    <sheet name="Data_Lenses" sheetId="36" state="hidden" r:id="rId36"/>
+    <sheet name="Data_MaterialChangeRollups" sheetId="37" state="hidden" r:id="rId37"/>
+    <sheet name="Data_OperatorOutcomes" sheetId="38" state="hidden" r:id="rId38"/>
+    <sheet name="Data_OperatorQueue" sheetId="39" state="hidden" r:id="rId39"/>
+    <sheet name="Data_OperatorRepoRollups" sheetId="40" state="hidden" r:id="rId40"/>
+    <sheet name="Data_PortfolioCatalog" sheetId="41" state="hidden" r:id="rId41"/>
+    <sheet name="Data_PortfolioHistory" sheetId="42" state="hidden" r:id="rId42"/>
+    <sheet name="Data_RepoDetail" sheetId="43" state="hidden" r:id="rId43"/>
+    <sheet name="Data_RepoDimensionRollups" sheetId="44" state="hidden" r:id="rId44"/>
+    <sheet name="Data_RepoHistoryRollups" sheetId="45" state="hidden" r:id="rId45"/>
+    <sheet name="Data_Repos" sheetId="46" state="hidden" r:id="rId46"/>
+    <sheet name="Data_ReviewHistory" sheetId="47" state="hidden" r:id="rId47"/>
+    <sheet name="Data_ReviewTargets" sheetId="48" state="hidden" r:id="rId48"/>
+    <sheet name="Data_Rollups" sheetId="49" state="hidden" r:id="rId49"/>
+    <sheet name="Data_RunChangeRepoData" sheetId="50" state="hidden" r:id="rId50"/>
+    <sheet name="Data_RunChangeRollups" sheetId="51" state="hidden" r:id="rId51"/>
+    <sheet name="Data_Scenarios" sheetId="52" state="hidden" r:id="rId52"/>
+    <sheet name="Data_Scorecards" sheetId="53" state="hidden" r:id="rId53"/>
+    <sheet name="Data_Security" sheetId="54" state="hidden" r:id="rId54"/>
+    <sheet name="Data_SecurityAlerts" sheetId="55" state="hidden" r:id="rId55"/>
+    <sheet name="Data_SecurityControls" sheetId="56" state="hidden" r:id="rId56"/>
+    <sheet name="Data_SecurityProviders" sheetId="57" state="hidden" r:id="rId57"/>
+    <sheet name="Data_TrendMatrix" sheetId="58" state="hidden" r:id="rId58"/>
+    <sheet name="Data_Writeback" sheetId="59" state="hidden" r:id="rId59"/>
+    <sheet name="Dep Graph" sheetId="60" state="hidden" r:id="rId60"/>
+    <sheet name="Governance Audit" sheetId="61" state="hidden" r:id="rId61"/>
+    <sheet name="Hotspots" sheetId="62" state="hidden" r:id="rId62"/>
+    <sheet name="Initiative Tracker" sheetId="63" state="hidden" r:id="rId63"/>
+    <sheet name="Lookups" sheetId="64" state="hidden" r:id="rId64"/>
+    <sheet name="Portfolio Catalog" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="Quick Wins" sheetId="66" state="hidden" r:id="rId66"/>
+    <sheet name="Repo Profiles" sheetId="67" state="hidden" r:id="rId67"/>
+    <sheet name="Review History" sheetId="68" state="hidden" r:id="rId68"/>
+    <sheet name="Scenario Planner" sheetId="69" state="hidden" r:id="rId69"/>
+    <sheet name="Score Explainer" sheetId="70" state="hidden" r:id="rId70"/>
+    <sheet name="Scorecards" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="Scoring Heatmap" sheetId="72" state="hidden" r:id="rId72"/>
+    <sheet name="Security" sheetId="73" state="hidden" r:id="rId73"/>
+    <sheet name="Security Controls" sheetId="74" state="hidden" r:id="rId74"/>
+    <sheet name="Security Debt" sheetId="75" state="hidden" r:id="rId75"/>
+    <sheet name="Supply Chain" sheetId="76" state="hidden" r:id="rId76"/>
+    <sheet name="TemplateInfo" sheetId="77" state="hidden" r:id="rId77"/>
+    <sheet name="Tier Breakdown" sheetId="78" state="hidden" r:id="rId78"/>
+    <sheet name="Trends" sheetId="79" state="hidden" r:id="rId79"/>
+    <sheet name="Writeback Audit" sheetId="80" state="hidden" r:id="rId80"/>
   </sheets>
   <definedNames>
     <definedName name="nrGeneratedAt">'Dashboard'!$A$2</definedName>
@@ -721,14 +721,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -746,17 +746,17 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <dPt>
             <idx val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="166534"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -764,10 +764,10 @@
           <dPt>
             <idx val="1"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="1565C0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -775,10 +775,10 @@
           <dPt>
             <idx val="2"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D97706"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -786,10 +786,10 @@
           <dPt>
             <idx val="3"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C2410C"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -797,10 +797,10 @@
           <dPt>
             <idx val="4"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="6B7280"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -833,14 +833,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -859,7 +859,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -911,14 +911,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -937,7 +937,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -989,14 +989,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1013,7 +1013,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1021,7 +1021,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1031,7 +1031,7 @@
           <idx val="1"/>
           <order val="1"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+            <a:ln w="12700">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -1041,7 +1041,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1051,7 +1051,7 @@
           <idx val="2"/>
           <order val="2"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+            <a:ln w="12700">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -1061,7 +1061,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1082,8 +1082,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1110,8 +1110,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1137,14 +1137,14 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1163,10 +1163,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="7C3AED"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1218,14 +1218,14 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="26"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1248,14 +1248,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1280,14 +1280,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1312,14 +1312,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1372,7 +1372,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -1387,9 +1387,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1409,9 +1409,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1431,9 +1431,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1453,9 +1453,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1465,7 +1465,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1480,9 +1480,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1492,7 +1492,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -1507,9 +1507,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>